<commit_message>
update charts for exp 1 and exp 2&3
</commit_message>
<xml_diff>
--- a/report/models/dev_v1_original_model_comparison.xlsx
+++ b/report/models/dev_v1_original_model_comparison.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vnpnk\Documents\TUM\studies\semester 2\Terminology translation\terminology-translation\report\models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A984F40-6545-4E38-8B92-9FDD84BE7DC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03A30ADF-B3F1-4184-8DA1-1C2F224D4F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1440" yWindow="1008" windowWidth="21600" windowHeight="11232" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="metrics" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="25">
   <si>
     <t>mode</t>
   </si>
@@ -89,6 +89,15 @@
   <si>
     <t>data</t>
   </si>
+  <si>
+    <t>Qwen 3B base</t>
+  </si>
+  <si>
+    <t>Qwen 7B base</t>
+  </si>
+  <si>
+    <t>Qwen 7B lora 2ep</t>
+  </si>
 </sst>
 </file>
 
@@ -123,7 +132,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -178,8 +187,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="25">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -233,26 +248,6 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -320,17 +315,6 @@
       <bottom style="medium">
         <color rgb="FF000000"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -463,11 +447,74 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -478,191 +525,234 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -976,46 +1066,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="79" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="62" t="s">
+      <c r="B1" s="79" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="62" t="s">
+      <c r="C1" s="79" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="65"/>
-      <c r="G1" s="62" t="s">
+      <c r="D1" s="80"/>
+      <c r="E1" s="80"/>
+      <c r="F1" s="81"/>
+      <c r="G1" s="79" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="65"/>
-      <c r="K1" s="62" t="s">
+      <c r="H1" s="80"/>
+      <c r="I1" s="80"/>
+      <c r="J1" s="81"/>
+      <c r="K1" s="79" t="s">
         <v>4</v>
       </c>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="65"/>
-      <c r="O1" s="62" t="s">
+      <c r="L1" s="80"/>
+      <c r="M1" s="80"/>
+      <c r="N1" s="81"/>
+      <c r="O1" s="79" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="64"/>
-      <c r="Q1" s="64"/>
-      <c r="R1" s="65"/>
-      <c r="S1" s="62" t="s">
+      <c r="P1" s="80"/>
+      <c r="Q1" s="80"/>
+      <c r="R1" s="81"/>
+      <c r="S1" s="79" t="s">
         <v>6</v>
       </c>
-      <c r="T1" s="64"/>
-      <c r="U1" s="64"/>
-      <c r="V1" s="65"/>
+      <c r="T1" s="80"/>
+      <c r="U1" s="80"/>
+      <c r="V1" s="81"/>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A2" s="67"/>
-      <c r="B2" s="67"/>
+      <c r="A2" s="78"/>
+      <c r="B2" s="78"/>
       <c r="C2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1078,7 +1168,7 @@
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A3" s="66" t="s">
+      <c r="A3" s="76" t="s">
         <v>11</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -1122,7 +1212,7 @@
       <c r="V3" s="2"/>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A4" s="61"/>
+      <c r="A4" s="77"/>
       <c r="B4" s="2" t="s">
         <v>13</v>
       </c>
@@ -1164,7 +1254,7 @@
       <c r="V4" s="2"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A5" s="67"/>
+      <c r="A5" s="78"/>
       <c r="B5" s="4" t="s">
         <v>14</v>
       </c>
@@ -1206,7 +1296,7 @@
       <c r="V5" s="4"/>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A6" s="66" t="s">
+      <c r="A6" s="76" t="s">
         <v>15</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -1274,7 +1364,7 @@
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A7" s="61"/>
+      <c r="A7" s="77"/>
       <c r="B7" s="2" t="s">
         <v>13</v>
       </c>
@@ -1340,7 +1430,7 @@
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A8" s="67"/>
+      <c r="A8" s="78"/>
       <c r="B8" s="4" t="s">
         <v>14</v>
       </c>
@@ -1406,7 +1496,7 @@
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A9" s="66" t="s">
+      <c r="A9" s="76" t="s">
         <v>16</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -1474,7 +1564,7 @@
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A10" s="61"/>
+      <c r="A10" s="77"/>
       <c r="B10" s="2" t="s">
         <v>13</v>
       </c>
@@ -1540,7 +1630,7 @@
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A11" s="67"/>
+      <c r="A11" s="78"/>
       <c r="B11" s="4" t="s">
         <v>14</v>
       </c>
@@ -1628,46 +1718,46 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="85" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="62" t="s">
+      <c r="B1" s="79" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="62" t="s">
+      <c r="C1" s="79" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="65"/>
-      <c r="G1" s="62" t="s">
+      <c r="D1" s="80"/>
+      <c r="E1" s="80"/>
+      <c r="F1" s="81"/>
+      <c r="G1" s="79" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="65"/>
-      <c r="K1" s="62" t="s">
+      <c r="H1" s="80"/>
+      <c r="I1" s="80"/>
+      <c r="J1" s="81"/>
+      <c r="K1" s="79" t="s">
         <v>4</v>
       </c>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="65"/>
-      <c r="O1" s="62" t="s">
+      <c r="L1" s="80"/>
+      <c r="M1" s="80"/>
+      <c r="N1" s="81"/>
+      <c r="O1" s="79" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="64"/>
-      <c r="Q1" s="64"/>
-      <c r="R1" s="65"/>
-      <c r="S1" s="62" t="s">
+      <c r="P1" s="80"/>
+      <c r="Q1" s="80"/>
+      <c r="R1" s="81"/>
+      <c r="S1" s="79" t="s">
         <v>6</v>
       </c>
-      <c r="T1" s="64"/>
-      <c r="U1" s="64"/>
-      <c r="V1" s="65"/>
+      <c r="T1" s="80"/>
+      <c r="U1" s="80"/>
+      <c r="V1" s="81"/>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A2" s="61"/>
-      <c r="B2" s="67"/>
+      <c r="A2" s="77"/>
+      <c r="B2" s="78"/>
       <c r="C2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1730,7 +1820,7 @@
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="82" t="s">
         <v>18</v>
       </c>
       <c r="B3" s="11" t="s">
@@ -1798,7 +1888,7 @@
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A4" s="69"/>
+      <c r="A4" s="83"/>
       <c r="B4" s="11" t="s">
         <v>13</v>
       </c>
@@ -1864,7 +1954,7 @@
       </c>
     </row>
     <row r="5" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="69"/>
+      <c r="A5" s="83"/>
       <c r="B5" s="12" t="s">
         <v>14</v>
       </c>
@@ -1930,7 +2020,7 @@
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A6" s="70" t="s">
+      <c r="A6" s="84" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="11" t="s">
@@ -1998,7 +2088,7 @@
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A7" s="69"/>
+      <c r="A7" s="83"/>
       <c r="B7" s="11" t="s">
         <v>13</v>
       </c>
@@ -2064,7 +2154,7 @@
       </c>
     </row>
     <row r="8" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="69"/>
+      <c r="A8" s="83"/>
       <c r="B8" s="12" t="s">
         <v>14</v>
       </c>
@@ -2130,7 +2220,7 @@
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A9" s="68" t="s">
+      <c r="A9" s="82" t="s">
         <v>19</v>
       </c>
       <c r="B9" s="11" t="s">
@@ -2198,7 +2288,7 @@
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A10" s="69"/>
+      <c r="A10" s="83"/>
       <c r="B10" s="11" t="s">
         <v>13</v>
       </c>
@@ -2264,7 +2354,7 @@
       </c>
     </row>
     <row r="11" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="69"/>
+      <c r="A11" s="83"/>
       <c r="B11" s="12" t="s">
         <v>14</v>
       </c>
@@ -2348,558 +2438,1035 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{370075A6-6178-4368-BF96-7705C11282C4}">
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.21875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="71" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="62" t="s">
+      <c r="B1" s="73" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="57" t="s">
+      <c r="C1" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="58"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="57" t="s">
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="75" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="58"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="57" t="s">
+      <c r="G1" s="64"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="58"/>
-      <c r="K1" s="59"/>
-      <c r="L1" s="57" t="s">
+      <c r="J1" s="64"/>
+      <c r="K1" s="65"/>
+      <c r="L1" s="63" t="s">
         <v>5</v>
       </c>
-      <c r="M1" s="58"/>
-      <c r="N1" s="59"/>
-      <c r="O1" s="57" t="s">
+      <c r="M1" s="64"/>
+      <c r="N1" s="65"/>
+      <c r="O1" s="63" t="s">
         <v>6</v>
       </c>
-      <c r="P1" s="58"/>
-      <c r="Q1" s="58"/>
+      <c r="P1" s="64"/>
+      <c r="Q1" s="66"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A2" s="61"/>
-      <c r="B2" s="63"/>
-      <c r="C2" s="23" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="24" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" s="23" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="H2" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="I2" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="J2" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="K2" s="24" t="s">
-        <v>9</v>
-      </c>
-      <c r="L2" s="23" t="s">
-        <v>7</v>
-      </c>
-      <c r="M2" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="N2" s="24" t="s">
-        <v>9</v>
-      </c>
-      <c r="O2" s="23" t="s">
-        <v>7</v>
-      </c>
-      <c r="P2" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="Q2" s="25" t="s">
-        <v>9</v>
+      <c r="A2" s="72"/>
+      <c r="B2" s="74"/>
+      <c r="C2" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="57" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="57" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="57" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="58" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="J2" s="57" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" s="57" t="s">
+        <v>23</v>
+      </c>
+      <c r="L2" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="M2" s="57" t="s">
+        <v>22</v>
+      </c>
+      <c r="N2" s="57" t="s">
+        <v>23</v>
+      </c>
+      <c r="O2" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="P2" s="57" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q2" s="58" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A3" s="53" t="s">
+      <c r="A3" s="67" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="36">
+      <c r="C3" s="32">
         <v>48.603953464788439</v>
       </c>
-      <c r="D3" s="36">
+      <c r="D3" s="32">
         <v>30.314341825072031</v>
       </c>
-      <c r="E3" s="36">
+      <c r="E3" s="32">
         <v>36.272022745581957</v>
       </c>
-      <c r="F3" s="35">
+      <c r="F3" s="31">
         <v>73.959159052304628</v>
       </c>
-      <c r="G3" s="36">
+      <c r="G3" s="32">
         <v>61.292040764243417</v>
       </c>
-      <c r="H3" s="37">
+      <c r="H3" s="33">
         <v>66.127364361970223</v>
       </c>
-      <c r="I3" s="36">
+      <c r="I3" s="32">
         <v>60.470085470085458</v>
       </c>
-      <c r="J3" s="36">
+      <c r="J3" s="32">
         <v>43.803418803418801</v>
       </c>
-      <c r="K3" s="36">
+      <c r="K3" s="32">
         <v>51.495726495726487</v>
       </c>
-      <c r="L3" s="35">
+      <c r="L3" s="31">
         <v>0.89693990427473047</v>
       </c>
-      <c r="M3" s="36">
+      <c r="M3" s="32">
         <v>0.88991780066808046</v>
       </c>
-      <c r="N3" s="36">
+      <c r="N3" s="32">
         <v>0.89674815355106496</v>
       </c>
-      <c r="O3" s="35">
+      <c r="O3" s="31">
         <v>0.80610412926391584</v>
       </c>
-      <c r="P3" s="36">
+      <c r="P3" s="32">
         <v>0.782764811490127</v>
       </c>
-      <c r="Q3" s="37">
+      <c r="Q3" s="33">
         <v>0.80251346499102427</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A4" s="54"/>
-      <c r="B4" s="42" t="s">
+      <c r="A4" s="68"/>
+      <c r="B4" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="20">
+      <c r="C4" s="59">
         <v>35.787894341325583</v>
       </c>
-      <c r="D4" s="20">
+      <c r="D4" s="59">
         <v>14.651169789357709</v>
       </c>
-      <c r="E4" s="20">
+      <c r="E4" s="59">
         <v>30.02831440175181</v>
       </c>
-      <c r="F4" s="26">
+      <c r="F4" s="22">
         <v>66.592954990214764</v>
       </c>
-      <c r="G4" s="20">
+      <c r="G4" s="59">
         <v>36.540912400601911</v>
       </c>
-      <c r="H4" s="27">
+      <c r="H4" s="23">
         <v>59.123833504180467</v>
       </c>
-      <c r="I4" s="20">
+      <c r="I4" s="59">
         <v>70.270270270270274</v>
       </c>
-      <c r="J4" s="20">
+      <c r="J4" s="59">
         <v>53.783783783783782</v>
       </c>
-      <c r="K4" s="20">
+      <c r="K4" s="59">
         <v>67.567567567567565</v>
       </c>
-      <c r="L4" s="26">
+      <c r="L4" s="22">
         <v>0.89185199970822571</v>
       </c>
-      <c r="M4" s="20">
+      <c r="M4" s="59">
         <v>0.87760758741503286</v>
       </c>
-      <c r="N4" s="20">
+      <c r="N4" s="59">
         <v>0.88499734334137414</v>
       </c>
-      <c r="O4" s="26">
+      <c r="O4" s="22">
         <v>0.70406189555125698</v>
       </c>
-      <c r="P4" s="20">
+      <c r="P4" s="59">
         <v>0.66731141199226185</v>
       </c>
-      <c r="Q4" s="27">
+      <c r="Q4" s="23">
         <v>0.67698259187620868</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A5" s="54"/>
-      <c r="B5" s="43" t="s">
+      <c r="A5" s="68"/>
+      <c r="B5" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="44">
+      <c r="C5" s="40">
         <v>54.043411284350753</v>
       </c>
-      <c r="D5" s="44">
+      <c r="D5" s="40">
         <v>39.710501968462196</v>
       </c>
-      <c r="E5" s="44">
+      <c r="E5" s="40">
         <v>47.894235828028599</v>
       </c>
-      <c r="F5" s="45">
+      <c r="F5" s="41">
         <v>75.472381082722563</v>
       </c>
-      <c r="G5" s="44">
+      <c r="G5" s="40">
         <v>65.24327258597117</v>
       </c>
-      <c r="H5" s="46">
+      <c r="H5" s="42">
         <v>71.655896059788589</v>
       </c>
-      <c r="I5" s="44">
+      <c r="I5" s="40">
         <v>89.017341040462426</v>
       </c>
-      <c r="J5" s="44">
+      <c r="J5" s="40">
         <v>82.369942196531781</v>
       </c>
-      <c r="K5" s="44">
+      <c r="K5" s="40">
         <v>84.682080924855498</v>
       </c>
-      <c r="L5" s="45">
+      <c r="L5" s="41">
         <v>0.90548329683586992</v>
       </c>
-      <c r="M5" s="44">
+      <c r="M5" s="40">
         <v>0.88880971834277478</v>
       </c>
-      <c r="N5" s="44">
+      <c r="N5" s="40">
         <v>0.90711668271781065</v>
       </c>
-      <c r="O5" s="45">
+      <c r="O5" s="41">
         <v>0.80426356589147308</v>
       </c>
-      <c r="P5" s="44">
+      <c r="P5" s="40">
         <v>0.76356589147286835</v>
       </c>
-      <c r="Q5" s="46">
+      <c r="Q5" s="42">
         <v>0.80232558139534915</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A6" s="55" t="s">
+      <c r="A6" s="69" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="41" t="s">
+      <c r="B6" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="47">
+      <c r="C6" s="43">
         <v>53.145335580867503</v>
       </c>
-      <c r="D6" s="47">
+      <c r="D6" s="43">
         <v>35.351302616962627</v>
       </c>
-      <c r="E6" s="47">
+      <c r="E6" s="43">
         <v>40.7526662444401</v>
       </c>
-      <c r="F6" s="48">
+      <c r="F6" s="44">
         <v>77.622562682716335</v>
       </c>
-      <c r="G6" s="47">
+      <c r="G6" s="43">
         <v>67.49950716527168</v>
       </c>
-      <c r="H6" s="49">
+      <c r="H6" s="45">
         <v>70.864105194278082</v>
       </c>
-      <c r="I6" s="50">
+      <c r="I6" s="46">
         <v>74.98295841854123</v>
       </c>
-      <c r="J6" s="50">
+      <c r="J6" s="46">
         <v>67.416496250852077</v>
       </c>
-      <c r="K6" s="50">
+      <c r="K6" s="46">
         <v>70.381731424676204</v>
       </c>
-      <c r="L6" s="51">
+      <c r="L6" s="47">
         <v>0.9444055155334643</v>
       </c>
-      <c r="M6" s="50">
+      <c r="M6" s="46">
         <v>0.93289548872839945</v>
       </c>
-      <c r="N6" s="50">
+      <c r="N6" s="46">
         <v>0.94022851514187056</v>
       </c>
-      <c r="O6" s="51">
+      <c r="O6" s="47">
         <v>0.86347724620770194</v>
       </c>
-      <c r="P6" s="50">
+      <c r="P6" s="46">
         <v>0.83663943990665057</v>
       </c>
-      <c r="Q6" s="52">
+      <c r="Q6" s="48">
         <v>0.85530921820303463</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A7" s="54"/>
-      <c r="B7" s="42" t="s">
+      <c r="A7" s="68"/>
+      <c r="B7" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="21">
+      <c r="C7" s="60">
         <v>43.14643446007593</v>
       </c>
-      <c r="D7" s="21">
+      <c r="D7" s="60">
         <v>24.502516891990421</v>
       </c>
-      <c r="E7" s="21">
+      <c r="E7" s="60">
         <v>37.86997424719835</v>
       </c>
-      <c r="F7" s="28">
+      <c r="F7" s="24">
         <v>72.496076334936589</v>
       </c>
-      <c r="G7" s="21">
+      <c r="G7" s="60">
         <v>51.439742043686188</v>
       </c>
-      <c r="H7" s="29">
+      <c r="H7" s="25">
         <v>66.917613939646841</v>
       </c>
-      <c r="I7" s="22">
+      <c r="I7" s="61">
         <v>79.418604651162795</v>
       </c>
-      <c r="J7" s="21">
+      <c r="J7" s="60">
         <v>63.255813953488371</v>
       </c>
-      <c r="K7" s="22">
+      <c r="K7" s="61">
         <v>77.20930232558139</v>
       </c>
-      <c r="L7" s="30">
+      <c r="L7" s="26">
         <v>0.94108656539680224</v>
       </c>
-      <c r="M7" s="22">
+      <c r="M7" s="61">
         <v>0.92936778771211703</v>
       </c>
-      <c r="N7" s="22">
+      <c r="N7" s="61">
         <v>0.93378162227790551</v>
       </c>
-      <c r="O7" s="30">
+      <c r="O7" s="26">
         <v>0.79054916985951484</v>
       </c>
-      <c r="P7" s="22">
+      <c r="P7" s="61">
         <v>0.75095785440613139</v>
       </c>
-      <c r="Q7" s="31">
+      <c r="Q7" s="27">
         <v>0.77139208173690865</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A8" s="54"/>
-      <c r="B8" s="43" t="s">
+      <c r="A8" s="68"/>
+      <c r="B8" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="40">
+      <c r="C8" s="36">
         <v>65.500393974696436</v>
       </c>
-      <c r="D8" s="40">
+      <c r="D8" s="36">
         <v>53.025648889320728</v>
       </c>
-      <c r="E8" s="40">
+      <c r="E8" s="36">
         <v>60.713459452875547</v>
       </c>
-      <c r="F8" s="38">
+      <c r="F8" s="34">
         <v>82.237677951785201</v>
       </c>
-      <c r="G8" s="40">
+      <c r="G8" s="36">
         <v>74.206038879449949</v>
       </c>
-      <c r="H8" s="39">
+      <c r="H8" s="35">
         <v>79.391221854359117</v>
       </c>
-      <c r="I8" s="33">
+      <c r="I8" s="29">
         <v>93.164794007490642</v>
       </c>
-      <c r="J8" s="40">
+      <c r="J8" s="36">
         <v>84.644194756554299</v>
       </c>
-      <c r="K8" s="33">
+      <c r="K8" s="29">
         <v>91.198501872659179</v>
       </c>
-      <c r="L8" s="32">
+      <c r="L8" s="28">
         <v>0.95926260542867181</v>
       </c>
-      <c r="M8" s="33">
+      <c r="M8" s="29">
         <v>0.95241161699079802</v>
       </c>
-      <c r="N8" s="33">
+      <c r="N8" s="29">
         <v>0.95719281356733632</v>
       </c>
-      <c r="O8" s="32">
+      <c r="O8" s="28">
         <v>0.87352625937834816</v>
       </c>
-      <c r="P8" s="33">
+      <c r="P8" s="29">
         <v>0.85101822079314049</v>
       </c>
-      <c r="Q8" s="34">
+      <c r="Q8" s="30">
         <v>0.87031082529474713</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A9" s="56" t="s">
+      <c r="A9" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="42" t="s">
+      <c r="B9" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="61">
         <v>51.244445997833303</v>
       </c>
-      <c r="D9" s="22">
+      <c r="D9" s="61">
         <v>32.319174933110382</v>
       </c>
-      <c r="E9" s="22">
+      <c r="E9" s="61">
         <v>36.2882873129007</v>
       </c>
-      <c r="F9" s="30">
+      <c r="F9" s="26">
         <v>75.695445305987207</v>
       </c>
-      <c r="G9" s="22">
+      <c r="G9" s="61">
         <v>64.254647584241781</v>
       </c>
-      <c r="H9" s="31">
+      <c r="H9" s="27">
         <v>67.48956991652733</v>
       </c>
-      <c r="I9" s="21">
+      <c r="I9" s="60">
         <v>80.208333333333343</v>
       </c>
-      <c r="J9" s="21">
+      <c r="J9" s="60">
         <v>72.8125</v>
       </c>
-      <c r="K9" s="21">
+      <c r="K9" s="60">
         <v>72.34375</v>
       </c>
-      <c r="L9" s="28">
+      <c r="L9" s="24">
         <v>0.97884245414673043</v>
       </c>
-      <c r="M9" s="21">
+      <c r="M9" s="60">
         <v>0.97748006379585317</v>
       </c>
-      <c r="N9" s="21">
+      <c r="N9" s="60">
         <v>0.97457162081339699</v>
       </c>
-      <c r="O9" s="28">
+      <c r="O9" s="24">
         <v>0.94930875576036888</v>
       </c>
-      <c r="P9" s="21">
+      <c r="P9" s="60">
         <v>0.94470046082949333</v>
       </c>
-      <c r="Q9" s="29">
+      <c r="Q9" s="25">
         <v>0.94009216589861777</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A10" s="54"/>
-      <c r="B10" s="42" t="s">
+      <c r="A10" s="68"/>
+      <c r="B10" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="22">
+      <c r="C10" s="61">
         <v>39.220045862976157</v>
       </c>
-      <c r="D10" s="22">
+      <c r="D10" s="61">
         <v>22.150691416062131</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="61">
         <v>34.153327663625603</v>
       </c>
-      <c r="F10" s="30">
+      <c r="F10" s="26">
         <v>68.370850450323445</v>
       </c>
-      <c r="G10" s="22">
+      <c r="G10" s="61">
         <v>48.666518965472576</v>
       </c>
-      <c r="H10" s="31">
+      <c r="H10" s="27">
         <v>62.693279966521423</v>
       </c>
-      <c r="I10" s="21">
+      <c r="I10" s="60">
         <v>79.602888086642594</v>
       </c>
-      <c r="J10" s="22">
+      <c r="J10" s="61">
         <v>62.635379061371843</v>
       </c>
-      <c r="K10" s="21">
+      <c r="K10" s="60">
         <v>77.978339350180505</v>
       </c>
-      <c r="L10" s="28">
+      <c r="L10" s="24">
         <v>0.96797396346132802</v>
       </c>
-      <c r="M10" s="21">
+      <c r="M10" s="60">
         <v>0.96674324472158391</v>
       </c>
-      <c r="N10" s="21">
+      <c r="N10" s="60">
         <v>0.96917733289574459</v>
       </c>
-      <c r="O10" s="28">
+      <c r="O10" s="24">
         <v>0.912121212121212</v>
       </c>
-      <c r="P10" s="21">
+      <c r="P10" s="60">
         <v>0.90303030303030307</v>
       </c>
-      <c r="Q10" s="29">
+      <c r="Q10" s="25">
         <v>0.91212121212121211</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A11" s="54"/>
-      <c r="B11" s="43" t="s">
+      <c r="A11" s="68"/>
+      <c r="B11" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="33">
+      <c r="C11" s="29">
         <v>61.131163000942948</v>
       </c>
-      <c r="D11" s="33">
+      <c r="D11" s="29">
         <v>47.582481739165452</v>
       </c>
-      <c r="E11" s="33">
+      <c r="E11" s="29">
         <v>56.113481237563583</v>
       </c>
-      <c r="F11" s="32">
+      <c r="F11" s="28">
         <v>79.033546463360238</v>
       </c>
-      <c r="G11" s="33">
+      <c r="G11" s="29">
         <v>69.972063013186329</v>
       </c>
-      <c r="H11" s="34">
+      <c r="H11" s="30">
         <v>76.023768740315191</v>
       </c>
-      <c r="I11" s="40">
+      <c r="I11" s="36">
         <v>95.75070821529745</v>
       </c>
-      <c r="J11" s="33">
+      <c r="J11" s="29">
         <v>84.135977337110475</v>
       </c>
-      <c r="K11" s="40">
+      <c r="K11" s="36">
         <v>92.067988668555245</v>
       </c>
-      <c r="L11" s="38">
+      <c r="L11" s="34">
         <v>0.97247403210576011</v>
       </c>
-      <c r="M11" s="40">
+      <c r="M11" s="36">
         <v>0.97046404964251975</v>
       </c>
-      <c r="N11" s="40">
+      <c r="N11" s="36">
         <v>0.97200188857412639</v>
       </c>
-      <c r="O11" s="38">
+      <c r="O11" s="34">
         <v>0.92156862745098023</v>
       </c>
-      <c r="P11" s="40">
+      <c r="P11" s="36">
         <v>0.91503267973856217</v>
       </c>
-      <c r="Q11" s="39">
+      <c r="Q11" s="35">
         <v>0.92156862745098023</v>
       </c>
     </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A13" s="71" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="73" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" s="63" t="s">
+        <v>2</v>
+      </c>
+      <c r="D13" s="64"/>
+      <c r="E13" s="64"/>
+      <c r="F13" s="75" t="s">
+        <v>3</v>
+      </c>
+      <c r="G13" s="64"/>
+      <c r="H13" s="66"/>
+      <c r="I13" s="64" t="s">
+        <v>4</v>
+      </c>
+      <c r="J13" s="64"/>
+      <c r="K13" s="65"/>
+      <c r="L13" s="63" t="s">
+        <v>5</v>
+      </c>
+      <c r="M13" s="64"/>
+      <c r="N13" s="65"/>
+      <c r="O13" s="63" t="s">
+        <v>6</v>
+      </c>
+      <c r="P13" s="64"/>
+      <c r="Q13" s="66"/>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A14" s="72"/>
+      <c r="B14" s="74"/>
+      <c r="C14" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D14" s="57" t="s">
+        <v>23</v>
+      </c>
+      <c r="E14" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="F14" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="G14" s="57" t="s">
+        <v>23</v>
+      </c>
+      <c r="H14" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="I14" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="J14" s="57" t="s">
+        <v>23</v>
+      </c>
+      <c r="K14" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="L14" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="M14" s="57" t="s">
+        <v>23</v>
+      </c>
+      <c r="N14" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="O14" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="P14" s="57" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q14" s="58" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A15" s="67" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="37" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="49">
+        <v>48.603953464788439</v>
+      </c>
+      <c r="D15" s="49">
+        <v>36.272022745581957</v>
+      </c>
+      <c r="E15" s="49"/>
+      <c r="F15" s="50">
+        <v>73.959159052304628</v>
+      </c>
+      <c r="G15" s="49">
+        <v>66.127364361970223</v>
+      </c>
+      <c r="H15" s="51"/>
+      <c r="I15" s="49">
+        <v>60.470085470085458</v>
+      </c>
+      <c r="J15" s="49">
+        <v>51.495726495726487</v>
+      </c>
+      <c r="K15" s="49"/>
+      <c r="L15" s="50">
+        <v>0.89693990427473047</v>
+      </c>
+      <c r="M15" s="49">
+        <v>0.89674815355106496</v>
+      </c>
+      <c r="N15" s="49"/>
+      <c r="O15" s="50">
+        <v>0.80610412926391584</v>
+      </c>
+      <c r="P15" s="49">
+        <v>0.80251346499102427</v>
+      </c>
+      <c r="Q15" s="51"/>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A16" s="68"/>
+      <c r="B16" s="38" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" s="62">
+        <v>35.787894341325583</v>
+      </c>
+      <c r="D16" s="62">
+        <v>30.02831440175181</v>
+      </c>
+      <c r="E16" s="62"/>
+      <c r="F16" s="52">
+        <v>66.592954990214764</v>
+      </c>
+      <c r="G16" s="62">
+        <v>59.123833504180467</v>
+      </c>
+      <c r="H16" s="53"/>
+      <c r="I16" s="62">
+        <v>70.270270270270274</v>
+      </c>
+      <c r="J16" s="62">
+        <v>67.567567567567565</v>
+      </c>
+      <c r="K16" s="62"/>
+      <c r="L16" s="52">
+        <v>0.89185199970822571</v>
+      </c>
+      <c r="M16" s="62">
+        <v>0.88499734334137414</v>
+      </c>
+      <c r="N16" s="62"/>
+      <c r="O16" s="52">
+        <v>0.70406189555125698</v>
+      </c>
+      <c r="P16" s="62">
+        <v>0.67698259187620868</v>
+      </c>
+      <c r="Q16" s="53"/>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A17" s="68"/>
+      <c r="B17" s="39" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="54">
+        <v>54.043411284350753</v>
+      </c>
+      <c r="D17" s="54">
+        <v>47.894235828028599</v>
+      </c>
+      <c r="E17" s="54"/>
+      <c r="F17" s="55">
+        <v>75.472381082722563</v>
+      </c>
+      <c r="G17" s="54">
+        <v>71.655896059788589</v>
+      </c>
+      <c r="H17" s="56"/>
+      <c r="I17" s="54">
+        <v>89.017341040462426</v>
+      </c>
+      <c r="J17" s="54">
+        <v>84.682080924855498</v>
+      </c>
+      <c r="K17" s="54"/>
+      <c r="L17" s="55">
+        <v>0.90548329683586992</v>
+      </c>
+      <c r="M17" s="54">
+        <v>0.90711668271781065</v>
+      </c>
+      <c r="N17" s="54"/>
+      <c r="O17" s="55">
+        <v>0.80426356589147308</v>
+      </c>
+      <c r="P17" s="54">
+        <v>0.80232558139534915</v>
+      </c>
+      <c r="Q17" s="56"/>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A18" s="69" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="37" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="49">
+        <v>53.145335580867503</v>
+      </c>
+      <c r="D18" s="49">
+        <v>40.7526662444401</v>
+      </c>
+      <c r="E18" s="49"/>
+      <c r="F18" s="50">
+        <v>77.622562682716335</v>
+      </c>
+      <c r="G18" s="49">
+        <v>70.864105194278082</v>
+      </c>
+      <c r="H18" s="51"/>
+      <c r="I18" s="49">
+        <v>74.98295841854123</v>
+      </c>
+      <c r="J18" s="49">
+        <v>70.381731424676204</v>
+      </c>
+      <c r="K18" s="49"/>
+      <c r="L18" s="50">
+        <v>0.9444055155334643</v>
+      </c>
+      <c r="M18" s="49">
+        <v>0.94022851514187056</v>
+      </c>
+      <c r="N18" s="49"/>
+      <c r="O18" s="50">
+        <v>0.86347724620770194</v>
+      </c>
+      <c r="P18" s="49">
+        <v>0.85530921820303463</v>
+      </c>
+      <c r="Q18" s="51"/>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A19" s="68"/>
+      <c r="B19" s="38" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="62">
+        <v>43.14643446007593</v>
+      </c>
+      <c r="D19" s="62">
+        <v>37.86997424719835</v>
+      </c>
+      <c r="E19" s="62"/>
+      <c r="F19" s="52">
+        <v>72.496076334936589</v>
+      </c>
+      <c r="G19" s="62">
+        <v>66.917613939646841</v>
+      </c>
+      <c r="H19" s="53"/>
+      <c r="I19" s="62">
+        <v>79.418604651162795</v>
+      </c>
+      <c r="J19" s="62">
+        <v>77.20930232558139</v>
+      </c>
+      <c r="K19" s="62"/>
+      <c r="L19" s="52">
+        <v>0.94108656539680224</v>
+      </c>
+      <c r="M19" s="62">
+        <v>0.93378162227790551</v>
+      </c>
+      <c r="N19" s="62"/>
+      <c r="O19" s="52">
+        <v>0.79054916985951484</v>
+      </c>
+      <c r="P19" s="62">
+        <v>0.77139208173690865</v>
+      </c>
+      <c r="Q19" s="53"/>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A20" s="68"/>
+      <c r="B20" s="39" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="54">
+        <v>65.500393974696436</v>
+      </c>
+      <c r="D20" s="54">
+        <v>60.713459452875547</v>
+      </c>
+      <c r="E20" s="54"/>
+      <c r="F20" s="55">
+        <v>82.237677951785201</v>
+      </c>
+      <c r="G20" s="54">
+        <v>79.391221854359117</v>
+      </c>
+      <c r="H20" s="56"/>
+      <c r="I20" s="54">
+        <v>93.164794007490642</v>
+      </c>
+      <c r="J20" s="54">
+        <v>91.198501872659179</v>
+      </c>
+      <c r="K20" s="54"/>
+      <c r="L20" s="55">
+        <v>0.95926260542867181</v>
+      </c>
+      <c r="M20" s="54">
+        <v>0.95719281356733632</v>
+      </c>
+      <c r="N20" s="54"/>
+      <c r="O20" s="55">
+        <v>0.87352625937834816</v>
+      </c>
+      <c r="P20" s="54">
+        <v>0.87031082529474713</v>
+      </c>
+      <c r="Q20" s="56"/>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A21" s="70" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="38" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="62">
+        <v>51.244445997833303</v>
+      </c>
+      <c r="D21" s="62">
+        <v>36.2882873129007</v>
+      </c>
+      <c r="E21" s="62"/>
+      <c r="F21" s="52">
+        <v>75.695445305987207</v>
+      </c>
+      <c r="G21" s="62">
+        <v>67.48956991652733</v>
+      </c>
+      <c r="H21" s="53"/>
+      <c r="I21" s="62">
+        <v>80.208333333333343</v>
+      </c>
+      <c r="J21" s="62">
+        <v>72.34375</v>
+      </c>
+      <c r="K21" s="62"/>
+      <c r="L21" s="52">
+        <v>0.97884245414673043</v>
+      </c>
+      <c r="M21" s="62">
+        <v>0.97457162081339699</v>
+      </c>
+      <c r="N21" s="62"/>
+      <c r="O21" s="52">
+        <v>0.94930875576036888</v>
+      </c>
+      <c r="P21" s="62">
+        <v>0.94009216589861777</v>
+      </c>
+      <c r="Q21" s="53"/>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A22" s="68"/>
+      <c r="B22" s="38" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22" s="62">
+        <v>39.220045862976157</v>
+      </c>
+      <c r="D22" s="62">
+        <v>34.153327663625603</v>
+      </c>
+      <c r="E22" s="62"/>
+      <c r="F22" s="52">
+        <v>68.370850450323445</v>
+      </c>
+      <c r="G22" s="62">
+        <v>62.693279966521423</v>
+      </c>
+      <c r="H22" s="53"/>
+      <c r="I22" s="62">
+        <v>79.602888086642594</v>
+      </c>
+      <c r="J22" s="62">
+        <v>77.978339350180505</v>
+      </c>
+      <c r="K22" s="62"/>
+      <c r="L22" s="52">
+        <v>0.96797396346132802</v>
+      </c>
+      <c r="M22" s="62">
+        <v>0.96917733289574459</v>
+      </c>
+      <c r="N22" s="62"/>
+      <c r="O22" s="52">
+        <v>0.912121212121212</v>
+      </c>
+      <c r="P22" s="62">
+        <v>0.91212121212121211</v>
+      </c>
+      <c r="Q22" s="53"/>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A23" s="68"/>
+      <c r="B23" s="39" t="s">
+        <v>14</v>
+      </c>
+      <c r="C23" s="54">
+        <v>61.131163000942948</v>
+      </c>
+      <c r="D23" s="54">
+        <v>56.113481237563583</v>
+      </c>
+      <c r="E23" s="54"/>
+      <c r="F23" s="55">
+        <v>79.033546463360238</v>
+      </c>
+      <c r="G23" s="54">
+        <v>76.023768740315191</v>
+      </c>
+      <c r="H23" s="56"/>
+      <c r="I23" s="54">
+        <v>95.75070821529745</v>
+      </c>
+      <c r="J23" s="54">
+        <v>92.067988668555245</v>
+      </c>
+      <c r="K23" s="54"/>
+      <c r="L23" s="55">
+        <v>0.97247403210576011</v>
+      </c>
+      <c r="M23" s="54">
+        <v>0.97200188857412639</v>
+      </c>
+      <c r="N23" s="54"/>
+      <c r="O23" s="55">
+        <v>0.92156862745098023</v>
+      </c>
+      <c r="P23" s="54">
+        <v>0.92156862745098023</v>
+      </c>
+      <c r="Q23" s="56"/>
+    </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="20">
     <mergeCell ref="I1:K1"/>
     <mergeCell ref="L1:N1"/>
     <mergeCell ref="O1:Q1"/>
@@ -2910,6 +3477,16 @@
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="F1:H1"/>
+    <mergeCell ref="L13:N13"/>
+    <mergeCell ref="O13:Q13"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="F13:H13"/>
+    <mergeCell ref="I13:K13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>